<commit_message>
Save usna so I can use on mac
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O625"/>
+  <dimension ref="A1:O626"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -3899,7 +3899,7 @@
         <v>1063136</v>
       </c>
       <c r="E98">
-        <v>210658</v>
+        <v>210662</v>
       </c>
       <c r="F98">
         <v>15063795</v>
@@ -3908,7 +3908,7 @@
         <v>12152139</v>
       </c>
       <c r="H98">
-        <v>904864</v>
+        <v>904873</v>
       </c>
       <c r="I98">
         <v>104.65</v>
@@ -3923,13 +3923,13 @@
         <v>79.33</v>
       </c>
       <c r="M98">
-        <v>8643085</v>
+        <v>8643095</v>
       </c>
       <c r="N98">
         <v>7816720</v>
       </c>
       <c r="O98">
-        <v>2726122</v>
+        <v>2726126</v>
       </c>
     </row>
     <row r="99">
@@ -3967,13 +3967,13 @@
         <v>79.84</v>
       </c>
       <c r="M99">
-        <v>8586173</v>
+        <v>8586182</v>
       </c>
       <c r="N99">
         <v>7675188</v>
       </c>
       <c r="O99">
-        <v>2658762</v>
+        <v>2658766</v>
       </c>
     </row>
     <row r="100">
@@ -4011,13 +4011,13 @@
         <v>80.49</v>
       </c>
       <c r="M100">
-        <v>8552546</v>
+        <v>8552555</v>
       </c>
       <c r="N100">
         <v>7655474</v>
       </c>
       <c r="O100">
-        <v>2569592</v>
+        <v>2569596</v>
       </c>
     </row>
     <row r="101">
@@ -4055,13 +4055,13 @@
         <v>80.95</v>
       </c>
       <c r="M101">
-        <v>8496269</v>
+        <v>8496279</v>
       </c>
       <c r="N101">
         <v>7630816</v>
       </c>
       <c r="O101">
-        <v>2496708</v>
+        <v>2496712</v>
       </c>
     </row>
     <row r="102">
@@ -4099,13 +4099,13 @@
         <v>81.34999999999999</v>
       </c>
       <c r="M102">
-        <v>8469972</v>
+        <v>8469981</v>
       </c>
       <c r="N102">
         <v>7605385</v>
       </c>
       <c r="O102">
-        <v>2447764</v>
+        <v>2447768</v>
       </c>
     </row>
     <row r="103">
@@ -4143,13 +4143,13 @@
         <v>81.74</v>
       </c>
       <c r="M103">
-        <v>8390310</v>
+        <v>8390320</v>
       </c>
       <c r="N103">
         <v>7610191</v>
       </c>
       <c r="O103">
-        <v>2369797</v>
+        <v>2369801</v>
       </c>
     </row>
     <row r="104">
@@ -4187,13 +4187,13 @@
         <v>82.12000000000001</v>
       </c>
       <c r="M104">
-        <v>8353736</v>
+        <v>8353745</v>
       </c>
       <c r="N104">
         <v>7610967</v>
       </c>
       <c r="O104">
-        <v>2306250</v>
+        <v>2306254</v>
       </c>
     </row>
     <row r="105">
@@ -4228,16 +4228,16 @@
         <v>13.57</v>
       </c>
       <c r="L105">
-        <v>82.48</v>
+        <v>82.49</v>
       </c>
       <c r="M105">
-        <v>8358613</v>
+        <v>8358622</v>
       </c>
       <c r="N105">
         <v>7677889</v>
       </c>
       <c r="O105">
-        <v>2230963</v>
+        <v>2230967</v>
       </c>
     </row>
     <row r="106">
@@ -4275,13 +4275,13 @@
         <v>82.78</v>
       </c>
       <c r="M106">
-        <v>8313955</v>
+        <v>8313965</v>
       </c>
       <c r="N106">
         <v>7636142</v>
       </c>
       <c r="O106">
-        <v>2171021</v>
+        <v>2171025</v>
       </c>
     </row>
     <row r="107">
@@ -4319,13 +4319,13 @@
         <v>83.03</v>
       </c>
       <c r="M107">
-        <v>8307250</v>
+        <v>8307260</v>
       </c>
       <c r="N107">
         <v>7633029</v>
       </c>
       <c r="O107">
-        <v>2121249</v>
+        <v>2121253</v>
       </c>
     </row>
     <row r="108">
@@ -4363,13 +4363,13 @@
         <v>83.3</v>
       </c>
       <c r="M108">
-        <v>8263899</v>
+        <v>8263909</v>
       </c>
       <c r="N108">
         <v>7603593</v>
       </c>
       <c r="O108">
-        <v>2073374</v>
+        <v>2073378</v>
       </c>
     </row>
     <row r="109">
@@ -4407,13 +4407,13 @@
         <v>83.67</v>
       </c>
       <c r="M109">
-        <v>8212234</v>
+        <v>8212243</v>
       </c>
       <c r="N109">
         <v>7568310</v>
       </c>
       <c r="O109">
-        <v>2030436</v>
+        <v>2030440</v>
       </c>
     </row>
     <row r="110">
@@ -5404,7 +5404,7 @@
         <v>9516801</v>
       </c>
       <c r="H132">
-        <v>935101</v>
+        <v>935404</v>
       </c>
       <c r="I132">
         <v>94</v>
@@ -5419,7 +5419,7 @@
         <v>99.05</v>
       </c>
       <c r="M132">
-        <v>14066648</v>
+        <v>14066951</v>
       </c>
       <c r="N132">
         <v>9919645</v>
@@ -5463,7 +5463,7 @@
         <v>99.53</v>
       </c>
       <c r="M133">
-        <v>14469101</v>
+        <v>14469404</v>
       </c>
       <c r="N133">
         <v>9992123</v>
@@ -5504,10 +5504,10 @@
         <v>15.02</v>
       </c>
       <c r="L134">
-        <v>100.19</v>
+        <v>100.2</v>
       </c>
       <c r="M134">
-        <v>14604736</v>
+        <v>14605039</v>
       </c>
       <c r="N134">
         <v>9946214</v>
@@ -5551,7 +5551,7 @@
         <v>100.72</v>
       </c>
       <c r="M135">
-        <v>14690173</v>
+        <v>14690476</v>
       </c>
       <c r="N135">
         <v>9890722</v>
@@ -5592,10 +5592,10 @@
         <v>15.16</v>
       </c>
       <c r="L136">
-        <v>101.3</v>
+        <v>101.31</v>
       </c>
       <c r="M136">
-        <v>14866632</v>
+        <v>14866935</v>
       </c>
       <c r="N136">
         <v>9919839</v>
@@ -5639,7 +5639,7 @@
         <v>101.83</v>
       </c>
       <c r="M137">
-        <v>14861150</v>
+        <v>14861453</v>
       </c>
       <c r="N137">
         <v>9793604</v>
@@ -5680,10 +5680,10 @@
         <v>15.52</v>
       </c>
       <c r="L138">
-        <v>102.24</v>
+        <v>102.25</v>
       </c>
       <c r="M138">
-        <v>14670542</v>
+        <v>14670845</v>
       </c>
       <c r="N138">
         <v>9476838</v>
@@ -5727,7 +5727,7 @@
         <v>102.61</v>
       </c>
       <c r="M139">
-        <v>14466767</v>
+        <v>14467070</v>
       </c>
       <c r="N139">
         <v>9214474</v>
@@ -5744,7 +5744,7 @@
         <v>2112151</v>
       </c>
       <c r="D140">
-        <v>823650</v>
+        <v>823682</v>
       </c>
       <c r="E140">
         <v>246909</v>
@@ -5771,10 +5771,10 @@
         <v>103.08</v>
       </c>
       <c r="M140">
-        <v>14131547</v>
+        <v>14131850</v>
       </c>
       <c r="N140">
-        <v>8935486</v>
+        <v>8935518</v>
       </c>
       <c r="O140">
         <v>3281695</v>
@@ -5815,10 +5815,10 @@
         <v>103.59</v>
       </c>
       <c r="M141">
-        <v>13893843</v>
+        <v>13894146</v>
       </c>
       <c r="N141">
-        <v>8782001</v>
+        <v>8782033</v>
       </c>
       <c r="O141">
         <v>3240512</v>
@@ -5859,10 +5859,10 @@
         <v>104.14</v>
       </c>
       <c r="M142">
-        <v>13749750</v>
+        <v>13750053</v>
       </c>
       <c r="N142">
-        <v>8776269</v>
+        <v>8776301</v>
       </c>
       <c r="O142">
         <v>3193123</v>
@@ -5903,10 +5903,10 @@
         <v>104.75</v>
       </c>
       <c r="M143">
-        <v>13621619</v>
+        <v>13621922</v>
       </c>
       <c r="N143">
-        <v>8836711</v>
+        <v>8836743</v>
       </c>
       <c r="O143">
         <v>3101549</v>
@@ -5950,7 +5950,7 @@
         <v>13767328</v>
       </c>
       <c r="N144">
-        <v>9042519</v>
+        <v>9042551</v>
       </c>
       <c r="O144">
         <v>3043526</v>
@@ -5994,7 +5994,7 @@
         <v>14113290</v>
       </c>
       <c r="N145">
-        <v>9395139</v>
+        <v>9395171</v>
       </c>
       <c r="O145">
         <v>2989177</v>
@@ -6038,7 +6038,7 @@
         <v>14458798</v>
       </c>
       <c r="N146">
-        <v>9716003</v>
+        <v>9716035</v>
       </c>
       <c r="O146">
         <v>2937578</v>
@@ -6082,7 +6082,7 @@
         <v>14926884</v>
       </c>
       <c r="N147">
-        <v>9916834</v>
+        <v>9916866</v>
       </c>
       <c r="O147">
         <v>2929529</v>
@@ -6126,7 +6126,7 @@
         <v>15607688</v>
       </c>
       <c r="N148">
-        <v>10176467</v>
+        <v>10176499</v>
       </c>
       <c r="O148">
         <v>2979966</v>
@@ -6170,7 +6170,7 @@
         <v>16230878</v>
       </c>
       <c r="N149">
-        <v>10402048</v>
+        <v>10402080</v>
       </c>
       <c r="O149">
         <v>3052828</v>
@@ -6214,7 +6214,7 @@
         <v>16798094</v>
       </c>
       <c r="N150">
-        <v>10586448</v>
+        <v>10586480</v>
       </c>
       <c r="O150">
         <v>3145040</v>
@@ -6258,7 +6258,7 @@
         <v>17524614</v>
       </c>
       <c r="N151">
-        <v>10834361</v>
+        <v>10834393</v>
       </c>
       <c r="O151">
         <v>3279005</v>
@@ -7768,7 +7768,7 @@
         <v>1488338</v>
       </c>
       <c r="D186">
-        <v>590407</v>
+        <v>590488</v>
       </c>
       <c r="E186">
         <v>232183</v>
@@ -7780,7 +7780,7 @@
         <v>9067094</v>
       </c>
       <c r="H186">
-        <v>1209224</v>
+        <v>1209185</v>
       </c>
       <c r="I186">
         <v>126.92</v>
@@ -7795,10 +7795,10 @@
         <v>125.18</v>
       </c>
       <c r="M186">
-        <v>13890014</v>
+        <v>13889974</v>
       </c>
       <c r="N186">
-        <v>8211212</v>
+        <v>8211293</v>
       </c>
       <c r="O186">
         <v>2510371</v>
@@ -7839,10 +7839,10 @@
         <v>125.48</v>
       </c>
       <c r="M187">
-        <v>13966246</v>
+        <v>13966207</v>
       </c>
       <c r="N187">
-        <v>8231203</v>
+        <v>8231284</v>
       </c>
       <c r="O187">
         <v>2506811</v>
@@ -7883,10 +7883,10 @@
         <v>125.89</v>
       </c>
       <c r="M188">
-        <v>14177480</v>
+        <v>14177441</v>
       </c>
       <c r="N188">
-        <v>8310989</v>
+        <v>8311070</v>
       </c>
       <c r="O188">
         <v>2528409</v>
@@ -7927,10 +7927,10 @@
         <v>126.37</v>
       </c>
       <c r="M189">
-        <v>14260788</v>
+        <v>14260748</v>
       </c>
       <c r="N189">
-        <v>8315349</v>
+        <v>8315430</v>
       </c>
       <c r="O189">
         <v>2521451</v>
@@ -7947,7 +7947,7 @@
         <v>509987</v>
       </c>
       <c r="E190">
-        <v>181947</v>
+        <v>181946</v>
       </c>
       <c r="F190">
         <v>9164177</v>
@@ -7971,13 +7971,13 @@
         <v>126.79</v>
       </c>
       <c r="M190">
-        <v>14423115</v>
+        <v>14423076</v>
       </c>
       <c r="N190">
-        <v>8370930</v>
+        <v>8371011</v>
       </c>
       <c r="O190">
-        <v>2540060</v>
+        <v>2540059</v>
       </c>
     </row>
     <row r="191">
@@ -7988,10 +7988,10 @@
         <v>1667576</v>
       </c>
       <c r="D191">
-        <v>573527</v>
+        <v>573532</v>
       </c>
       <c r="E191">
-        <v>207676</v>
+        <v>207672</v>
       </c>
       <c r="F191">
         <v>9966680</v>
@@ -8000,7 +8000,7 @@
         <v>8715190</v>
       </c>
       <c r="H191">
-        <v>1072983</v>
+        <v>1073038</v>
       </c>
       <c r="I191">
         <v>129.49</v>
@@ -8015,13 +8015,13 @@
         <v>127.14</v>
       </c>
       <c r="M191">
-        <v>14528195</v>
+        <v>14528211</v>
       </c>
       <c r="N191">
-        <v>8368431</v>
+        <v>8368517</v>
       </c>
       <c r="O191">
-        <v>2551092</v>
+        <v>2551087</v>
       </c>
     </row>
     <row r="192">
@@ -8059,13 +8059,13 @@
         <v>127.59</v>
       </c>
       <c r="M192">
-        <v>14532969</v>
+        <v>14532986</v>
       </c>
       <c r="N192">
-        <v>8290005</v>
+        <v>8290091</v>
       </c>
       <c r="O192">
-        <v>2547714</v>
+        <v>2547709</v>
       </c>
     </row>
     <row r="193">
@@ -8103,13 +8103,13 @@
         <v>128.14</v>
       </c>
       <c r="M193">
-        <v>14761493</v>
+        <v>14761509</v>
       </c>
       <c r="N193">
-        <v>8365097</v>
+        <v>8365183</v>
       </c>
       <c r="O193">
-        <v>2572362</v>
+        <v>2572357</v>
       </c>
     </row>
     <row r="194">
@@ -8147,13 +8147,13 @@
         <v>128.88</v>
       </c>
       <c r="M194">
-        <v>14844174</v>
+        <v>14844190</v>
       </c>
       <c r="N194">
-        <v>8387984</v>
+        <v>8388070</v>
       </c>
       <c r="O194">
-        <v>2570162</v>
+        <v>2570157</v>
       </c>
     </row>
     <row r="195">
@@ -8191,13 +8191,13 @@
         <v>129.54</v>
       </c>
       <c r="M195">
-        <v>14889104</v>
+        <v>14889120</v>
       </c>
       <c r="N195">
-        <v>8325456</v>
+        <v>8325542</v>
       </c>
       <c r="O195">
-        <v>2571051</v>
+        <v>2571046</v>
       </c>
     </row>
     <row r="196">
@@ -8235,13 +8235,13 @@
         <v>130.2</v>
       </c>
       <c r="M196">
-        <v>14967786</v>
+        <v>14967802</v>
       </c>
       <c r="N196">
-        <v>8319952</v>
+        <v>8320038</v>
       </c>
       <c r="O196">
-        <v>2563125</v>
+        <v>2563120</v>
       </c>
     </row>
     <row r="197">
@@ -8279,13 +8279,13 @@
         <v>130.86</v>
       </c>
       <c r="M197">
-        <v>15089930</v>
+        <v>15089947</v>
       </c>
       <c r="N197">
-        <v>8341416</v>
+        <v>8341502</v>
       </c>
       <c r="O197">
-        <v>2566580</v>
+        <v>2566575</v>
       </c>
     </row>
     <row r="198">
@@ -8323,13 +8323,13 @@
         <v>131.55</v>
       </c>
       <c r="M198">
-        <v>15141431</v>
+        <v>15141487</v>
       </c>
       <c r="N198">
-        <v>8330287</v>
+        <v>8330292</v>
       </c>
       <c r="O198">
-        <v>2567381</v>
+        <v>2567376</v>
       </c>
     </row>
     <row r="199">
@@ -8343,7 +8343,7 @@
         <v>525103</v>
       </c>
       <c r="E199">
-        <v>214625</v>
+        <v>214628</v>
       </c>
       <c r="F199">
         <v>10193543</v>
@@ -8367,13 +8367,13 @@
         <v>132.19</v>
       </c>
       <c r="M199">
-        <v>15308975</v>
+        <v>15309031</v>
       </c>
       <c r="N199">
-        <v>8356535</v>
+        <v>8356540</v>
       </c>
       <c r="O199">
-        <v>2587930</v>
+        <v>2587928</v>
       </c>
     </row>
     <row r="200">
@@ -8387,7 +8387,7 @@
         <v>735606</v>
       </c>
       <c r="E200">
-        <v>247051</v>
+        <v>247052</v>
       </c>
       <c r="F200">
         <v>11601024</v>
@@ -8411,13 +8411,13 @@
         <v>132.87</v>
       </c>
       <c r="M200">
-        <v>15440585</v>
+        <v>15440640</v>
       </c>
       <c r="N200">
-        <v>8350554</v>
+        <v>8350559</v>
       </c>
       <c r="O200">
-        <v>2599983</v>
+        <v>2599982</v>
       </c>
     </row>
     <row r="201">
@@ -8452,16 +8452,16 @@
         <v>14.4</v>
       </c>
       <c r="L201">
-        <v>133.48</v>
+        <v>133.49</v>
       </c>
       <c r="M201">
-        <v>15510359</v>
+        <v>15510415</v>
       </c>
       <c r="N201">
-        <v>8368297</v>
+        <v>8368302</v>
       </c>
       <c r="O201">
-        <v>2605561</v>
+        <v>2605560</v>
       </c>
     </row>
     <row r="202">
@@ -8499,10 +8499,10 @@
         <v>134.04</v>
       </c>
       <c r="M202">
-        <v>15673669</v>
+        <v>15673725</v>
       </c>
       <c r="N202">
-        <v>8381854</v>
+        <v>8381859</v>
       </c>
       <c r="O202">
         <v>2635473</v>
@@ -8549,7 +8549,7 @@
         <v>8380544</v>
       </c>
       <c r="O203">
-        <v>2650970</v>
+        <v>2650974</v>
       </c>
     </row>
     <row r="204">
@@ -8593,7 +8593,7 @@
         <v>8330361</v>
       </c>
       <c r="O204">
-        <v>2658792</v>
+        <v>2658796</v>
       </c>
     </row>
     <row r="205">
@@ -8637,7 +8637,7 @@
         <v>8360752</v>
       </c>
       <c r="O205">
-        <v>2687341</v>
+        <v>2687345</v>
       </c>
     </row>
     <row r="206">
@@ -8681,7 +8681,7 @@
         <v>8190399</v>
       </c>
       <c r="O206">
-        <v>2682395</v>
+        <v>2682399</v>
       </c>
     </row>
     <row r="207">
@@ -8725,7 +8725,7 @@
         <v>8167954</v>
       </c>
       <c r="O207">
-        <v>2694746</v>
+        <v>2694750</v>
       </c>
     </row>
     <row r="208">
@@ -8769,7 +8769,7 @@
         <v>8133267</v>
       </c>
       <c r="O208">
-        <v>2719329</v>
+        <v>2719333</v>
       </c>
     </row>
     <row r="209">
@@ -8813,7 +8813,7 @@
         <v>8038963</v>
       </c>
       <c r="O209">
-        <v>2707771</v>
+        <v>2707775</v>
       </c>
     </row>
     <row r="210">
@@ -8857,7 +8857,7 @@
         <v>7908330</v>
       </c>
       <c r="O210">
-        <v>2680336</v>
+        <v>2680340</v>
       </c>
     </row>
     <row r="211">
@@ -8901,7 +8901,7 @@
         <v>7873641</v>
       </c>
       <c r="O211">
-        <v>2671979</v>
+        <v>2671980</v>
       </c>
     </row>
     <row r="212">
@@ -26612,7 +26612,7 @@
         <v>43769</v>
       </c>
       <c r="B599">
-        <v>878358</v>
+        <v>878311</v>
       </c>
       <c r="C599">
         <v>1385.4</v>
@@ -26659,7 +26659,7 @@
         <v>43799</v>
       </c>
       <c r="B600">
-        <v>964408</v>
+        <v>964398</v>
       </c>
       <c r="C600">
         <v>1525.9</v>
@@ -26706,7 +26706,7 @@
         <v>43830</v>
       </c>
       <c r="B601">
-        <v>1366407</v>
+        <v>1366439</v>
       </c>
       <c r="C601">
         <v>1786.2</v>
@@ -26753,7 +26753,7 @@
         <v>43861</v>
       </c>
       <c r="B602">
-        <v>1215627</v>
+        <v>1215506</v>
       </c>
       <c r="C602">
         <v>2045.2</v>
@@ -26800,7 +26800,7 @@
         <v>43890</v>
       </c>
       <c r="B603">
-        <v>843175</v>
+        <v>843098</v>
       </c>
       <c r="C603">
         <v>2047.1</v>
@@ -26847,7 +26847,7 @@
         <v>43921</v>
       </c>
       <c r="B604">
-        <v>11768425</v>
+        <v>11763805</v>
       </c>
       <c r="C604">
         <v>2232.5</v>
@@ -26894,7 +26894,7 @@
         <v>43951</v>
       </c>
       <c r="B605">
-        <v>17624674</v>
+        <v>17606753</v>
       </c>
       <c r="C605">
         <v>17346.7</v>
@@ -26906,16 +26906,16 @@
         <v>206020</v>
       </c>
       <c r="F605">
-        <v>66075737</v>
+        <v>66031203</v>
       </c>
       <c r="G605">
-        <v>55690467</v>
+        <v>55683268</v>
       </c>
       <c r="H605">
         <v>18328670</v>
       </c>
       <c r="I605">
-        <v>334.29</v>
+        <v>334.3</v>
       </c>
       <c r="J605">
         <v>35.66</v>
@@ -26941,7 +26941,7 @@
         <v>43982</v>
       </c>
       <c r="B606">
-        <v>9279296</v>
+        <v>9273398</v>
       </c>
       <c r="C606">
         <v>18746</v>
@@ -26988,7 +26988,7 @@
         <v>44012</v>
       </c>
       <c r="B607">
-        <v>6646812</v>
+        <v>6640918</v>
       </c>
       <c r="C607">
         <v>17052.6</v>
@@ -27035,7 +27035,7 @@
         <v>44043</v>
       </c>
       <c r="B608">
-        <v>5939361</v>
+        <v>5932955</v>
       </c>
       <c r="C608">
         <v>16315.1</v>
@@ -27082,7 +27082,7 @@
         <v>44074</v>
       </c>
       <c r="B609">
-        <v>3743201</v>
+        <v>3739543</v>
       </c>
       <c r="C609">
         <v>14100.6</v>
@@ -27094,16 +27094,16 @@
         <v>1067709</v>
       </c>
       <c r="F609">
-        <v>63156496</v>
+        <v>63188394</v>
       </c>
       <c r="G609">
-        <v>56382477</v>
+        <v>56411415</v>
       </c>
       <c r="H609">
         <v>16352575</v>
       </c>
       <c r="I609">
-        <v>304.64</v>
+        <v>304.66</v>
       </c>
       <c r="J609">
         <v>80.70999999999999</v>
@@ -27129,7 +27129,7 @@
         <v>44104</v>
       </c>
       <c r="B610">
-        <v>3489601</v>
+        <v>3485891</v>
       </c>
       <c r="C610">
         <v>12431.1</v>
@@ -27176,7 +27176,7 @@
         <v>44135</v>
       </c>
       <c r="B611">
-        <v>3443574</v>
+        <v>3440134</v>
       </c>
       <c r="C611">
         <v>7612.8</v>
@@ -27223,7 +27223,7 @@
         <v>44165</v>
       </c>
       <c r="B612">
-        <v>3431761</v>
+        <v>3429538</v>
       </c>
       <c r="C612">
         <v>6136</v>
@@ -27270,7 +27270,7 @@
         <v>44196</v>
       </c>
       <c r="B613">
-        <v>4222043</v>
+        <v>4219889</v>
       </c>
       <c r="C613">
         <v>5655.4</v>
@@ -27317,25 +27317,25 @@
         <v>44227</v>
       </c>
       <c r="B614">
-        <v>4597503</v>
+        <v>4594918</v>
       </c>
       <c r="C614">
         <v>5366.6</v>
       </c>
       <c r="D614">
-        <v>910844</v>
+        <v>910845</v>
       </c>
       <c r="E614">
-        <v>821765</v>
+        <v>821766</v>
       </c>
       <c r="F614">
-        <v>22584976</v>
+        <v>22586280</v>
       </c>
       <c r="G614">
-        <v>17533693</v>
+        <v>17533723</v>
       </c>
       <c r="H614">
-        <v>5618359</v>
+        <v>5618369</v>
       </c>
       <c r="I614">
         <v>346.07</v>
@@ -27350,13 +27350,13 @@
         <v>318.91</v>
       </c>
       <c r="M614">
-        <v>146096649</v>
+        <v>146096658</v>
       </c>
       <c r="N614">
-        <v>31003379</v>
+        <v>31003380</v>
       </c>
       <c r="O614">
-        <v>12105825</v>
+        <v>12105826</v>
       </c>
     </row>
     <row r="615">
@@ -27364,25 +27364,25 @@
         <v>44255</v>
       </c>
       <c r="B615">
-        <v>3555489</v>
+        <v>3553419</v>
       </c>
       <c r="C615">
         <v>5029.5</v>
       </c>
       <c r="D615">
-        <v>766125</v>
+        <v>766126</v>
       </c>
       <c r="E615">
         <v>633206</v>
       </c>
       <c r="F615">
-        <v>18840926</v>
+        <v>18842134</v>
       </c>
       <c r="G615">
-        <v>15831126</v>
+        <v>15831135</v>
       </c>
       <c r="H615">
-        <v>5068153</v>
+        <v>5068157</v>
       </c>
       <c r="I615">
         <v>349.14</v>
@@ -27397,13 +27397,13 @@
         <v>318.78</v>
       </c>
       <c r="M615">
-        <v>148411755</v>
+        <v>148411768</v>
       </c>
       <c r="N615">
-        <v>31290074</v>
+        <v>31290076</v>
       </c>
       <c r="O615">
-        <v>12600384</v>
+        <v>12600385</v>
       </c>
     </row>
     <row r="616">
@@ -27411,7 +27411,7 @@
         <v>44286</v>
       </c>
       <c r="B616">
-        <v>4200510</v>
+        <v>4197753</v>
       </c>
       <c r="C616">
         <v>4460.9</v>
@@ -27444,13 +27444,13 @@
         <v>318.51</v>
       </c>
       <c r="M616">
-        <v>149866318</v>
+        <v>149866331</v>
       </c>
       <c r="N616">
-        <v>30430491</v>
+        <v>30430493</v>
       </c>
       <c r="O616">
-        <v>13044262</v>
+        <v>13044263</v>
       </c>
     </row>
     <row r="617">
@@ -27458,7 +27458,7 @@
         <v>44316</v>
       </c>
       <c r="B617">
-        <v>3139798</v>
+        <v>3131048</v>
       </c>
       <c r="C617">
         <v>4022.4</v>
@@ -27491,13 +27491,13 @@
         <v>317.26</v>
       </c>
       <c r="M617">
-        <v>135606287</v>
+        <v>135606300</v>
       </c>
       <c r="N617">
-        <v>19269456</v>
+        <v>19269458</v>
       </c>
       <c r="O617">
-        <v>13246974</v>
+        <v>13246975</v>
       </c>
     </row>
     <row r="618">
@@ -27505,7 +27505,7 @@
         <v>44347</v>
       </c>
       <c r="B618">
-        <v>2221329</v>
+        <v>2180777</v>
       </c>
       <c r="C618">
         <v>3591.2</v>
@@ -27538,13 +27538,13 @@
         <v>317.62</v>
       </c>
       <c r="M618">
-        <v>115810473</v>
+        <v>115810487</v>
       </c>
       <c r="N618">
-        <v>14265040</v>
+        <v>14265042</v>
       </c>
       <c r="O618">
-        <v>13354759</v>
+        <v>13354760</v>
       </c>
     </row>
     <row r="619">
@@ -27552,7 +27552,7 @@
         <v>44377</v>
       </c>
       <c r="B619">
-        <v>2301654</v>
+        <v>2290434</v>
       </c>
       <c r="C619">
         <v>3473.1</v>
@@ -27585,13 +27585,13 @@
         <v>321.48</v>
       </c>
       <c r="M619">
-        <v>97731783</v>
+        <v>97731796</v>
       </c>
       <c r="N619">
-        <v>11764464</v>
+        <v>11764466</v>
       </c>
       <c r="O619">
-        <v>13082692</v>
+        <v>13082693</v>
       </c>
     </row>
     <row r="620">
@@ -27599,7 +27599,7 @@
         <v>44408</v>
       </c>
       <c r="B620">
-        <v>2049168</v>
+        <v>2048833</v>
       </c>
       <c r="C620">
         <v>3413.7</v>
@@ -27632,13 +27632,13 @@
         <v>326.54</v>
       </c>
       <c r="M620">
-        <v>82596549</v>
+        <v>82596563</v>
       </c>
       <c r="N620">
-        <v>10199122</v>
+        <v>10199124</v>
       </c>
       <c r="O620">
-        <v>12419292</v>
+        <v>12419293</v>
       </c>
     </row>
     <row r="621">
@@ -27646,7 +27646,7 @@
         <v>44439</v>
       </c>
       <c r="B621">
-        <v>1504461</v>
+        <v>1504150</v>
       </c>
       <c r="C621">
         <v>2944.1</v>
@@ -27679,13 +27679,13 @@
         <v>333.27</v>
       </c>
       <c r="M621">
-        <v>69691423</v>
+        <v>69691437</v>
       </c>
       <c r="N621">
-        <v>9343638</v>
+        <v>9343640</v>
       </c>
       <c r="O621">
-        <v>11625864</v>
+        <v>11625865</v>
       </c>
     </row>
     <row r="622">
@@ -27693,16 +27693,16 @@
         <v>44469</v>
       </c>
       <c r="B622">
-        <v>1407225</v>
+        <v>1407016</v>
       </c>
       <c r="C622">
         <v>2479.4</v>
       </c>
       <c r="D622">
-        <v>478251</v>
+        <v>481655</v>
       </c>
       <c r="E622">
-        <v>305836</v>
+        <v>298251.6666666667</v>
       </c>
       <c r="F622">
         <v>10043831</v>
@@ -27711,7 +27711,7 @@
         <v>8099142</v>
       </c>
       <c r="H622">
-        <v>2686603</v>
+        <v>2694227</v>
       </c>
       <c r="I622">
         <v>352.13</v>
@@ -27723,16 +27723,16 @@
         <v>20.98</v>
       </c>
       <c r="L622">
-        <v>340.11</v>
+        <v>340.1</v>
       </c>
       <c r="M622">
-        <v>58992537</v>
+        <v>59000175</v>
       </c>
       <c r="N622">
-        <v>8910182</v>
+        <v>8913588</v>
       </c>
       <c r="O622">
-        <v>8848636</v>
+        <v>8850631</v>
       </c>
     </row>
     <row r="623">
@@ -27764,22 +27764,22 @@
         <v>350.31</v>
       </c>
       <c r="J623">
-        <v>34.88</v>
+        <v>34.89</v>
       </c>
       <c r="K623">
         <v>19.46</v>
       </c>
       <c r="L623">
-        <v>344.47</v>
+        <v>344.45</v>
       </c>
       <c r="M623">
-        <v>52922911</v>
+        <v>52930549</v>
       </c>
       <c r="N623">
-        <v>8502763</v>
+        <v>8506169</v>
       </c>
       <c r="O623">
-        <v>6721100</v>
+        <v>6723095</v>
       </c>
     </row>
     <row r="624">
@@ -27811,22 +27811,22 @@
         <v>364.76</v>
       </c>
       <c r="J624">
-        <v>39.28</v>
+        <v>39.29</v>
       </c>
       <c r="K624">
-        <v>18.55</v>
+        <v>18.54</v>
       </c>
       <c r="L624">
-        <v>347.35</v>
+        <v>347.33</v>
       </c>
       <c r="M624">
-        <v>48468496</v>
+        <v>48476134</v>
       </c>
       <c r="N624">
-        <v>8090253</v>
+        <v>8093659</v>
       </c>
       <c r="O624">
-        <v>5602809</v>
+        <v>5604804</v>
       </c>
     </row>
     <row r="625">
@@ -27834,28 +27834,28 @@
         <v>44561</v>
       </c>
       <c r="B625">
-        <v>1280012</v>
+        <v>1265017</v>
       </c>
       <c r="C625">
         <v>1632.8</v>
       </c>
       <c r="D625">
-        <v>417825</v>
+        <v>413315</v>
       </c>
       <c r="E625">
-        <v>274529</v>
+        <v>182399</v>
       </c>
       <c r="F625">
-        <v>7758919</v>
+        <v>7674269</v>
       </c>
       <c r="G625">
-        <v>6149407</v>
+        <v>6082444</v>
       </c>
       <c r="H625">
-        <v>2202553</v>
+        <v>2186036</v>
       </c>
       <c r="I625">
-        <v>374.88</v>
+        <v>376.27</v>
       </c>
       <c r="J625">
         <v>40.34</v>
@@ -27864,16 +27864,63 @@
         <v>17.8</v>
       </c>
       <c r="L625">
-        <v>349.75</v>
+        <v>349.77</v>
       </c>
       <c r="M625">
-        <v>44281581</v>
+        <v>44272701</v>
       </c>
       <c r="N625">
-        <v>7633009</v>
+        <v>7631905</v>
       </c>
       <c r="O625">
-        <v>4746190</v>
+        <v>4745752</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2">
+        <v>44592</v>
+      </c>
+      <c r="B626">
+        <v>1414633</v>
+      </c>
+      <c r="C626">
+        <v>1825.066666666667</v>
+      </c>
+      <c r="D626">
+        <v>526769</v>
+      </c>
+      <c r="E626">
+        <v>177875</v>
+      </c>
+      <c r="F626">
+        <v>9136815</v>
+      </c>
+      <c r="G626">
+        <v>6989873</v>
+      </c>
+      <c r="H626">
+        <v>2493510</v>
+      </c>
+      <c r="I626">
+        <v>390.15</v>
+      </c>
+      <c r="J626">
+        <v>40.22</v>
+      </c>
+      <c r="K626">
+        <v>17.29</v>
+      </c>
+      <c r="L626">
+        <v>352.65</v>
+      </c>
+      <c r="M626">
+        <v>41147842</v>
+      </c>
+      <c r="N626">
+        <v>7247829</v>
+      </c>
+      <c r="O626">
+        <v>4101861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
has haver back up and deflators sheet
this has haver back up workbook in data folder, haver back up r script, has delfators forecast sheet, and the updated fim script to pull in deflators
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R635"/>
+  <dimension ref="A1:R636"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -33736,28 +33736,28 @@
         <v>44712</v>
       </c>
       <c r="B630">
-        <v>859355</v>
+        <v>858243</v>
       </c>
       <c r="C630">
         <v>1349.6</v>
       </c>
       <c r="D630">
-        <v>313024</v>
+        <v>313021</v>
       </c>
       <c r="E630">
-        <v>125577</v>
+        <v>125552</v>
       </c>
       <c r="F630">
-        <v>5994282</v>
+        <v>5982003</v>
       </c>
       <c r="G630">
-        <v>4675798</v>
+        <v>4675812</v>
       </c>
       <c r="H630">
-        <v>1815114</v>
+        <v>1815116</v>
       </c>
       <c r="I630">
-        <v>397.15</v>
+        <v>397.16</v>
       </c>
       <c r="J630">
         <v>32.57</v>
@@ -33769,13 +33769,13 @@
         <v>367.89</v>
       </c>
       <c r="M630">
-        <v>31534204</v>
+        <v>31534206</v>
       </c>
       <c r="N630">
-        <v>5196524</v>
+        <v>5196521</v>
       </c>
       <c r="O630">
-        <v>2635187</v>
+        <v>2635162</v>
       </c>
       <c r="P630">
         <v>5258</v>
@@ -33792,28 +33792,28 @@
         <v>44742</v>
       </c>
       <c r="B631">
-        <v>937326</v>
+        <v>936213</v>
       </c>
       <c r="C631">
         <v>1297.8</v>
       </c>
       <c r="D631">
-        <v>327883</v>
+        <v>327875</v>
       </c>
       <c r="E631">
-        <v>106319</v>
+        <v>106283</v>
       </c>
       <c r="F631">
-        <v>5524780</v>
+        <v>5513046</v>
       </c>
       <c r="G631">
-        <v>4383369</v>
+        <v>4383367</v>
       </c>
       <c r="H631">
-        <v>1692387</v>
+        <v>1692379</v>
       </c>
       <c r="I631">
-        <v>394.63</v>
+        <v>394.65</v>
       </c>
       <c r="J631">
         <v>31.55</v>
@@ -33825,13 +33825,13 @@
         <v>372.77</v>
       </c>
       <c r="M631">
-        <v>29240146</v>
+        <v>29240140</v>
       </c>
       <c r="N631">
-        <v>4865411</v>
+        <v>4865400</v>
       </c>
       <c r="O631">
-        <v>2407560</v>
+        <v>2407499</v>
       </c>
       <c r="P631">
         <v>5238</v>
@@ -33860,7 +33860,7 @@
         <v>113474</v>
       </c>
       <c r="F632">
-        <v>6320919</v>
+        <v>6320944</v>
       </c>
       <c r="G632">
         <v>4667208</v>
@@ -33881,13 +33881,13 @@
         <v>377.44</v>
       </c>
       <c r="M632">
-        <v>27537812</v>
+        <v>27537806</v>
       </c>
       <c r="N632">
-        <v>4641774</v>
+        <v>4641763</v>
       </c>
       <c r="O632">
-        <v>2234769</v>
+        <v>2234708</v>
       </c>
       <c r="P632">
         <v>5246</v>
@@ -33904,46 +33904,46 @@
         <v>44804</v>
       </c>
       <c r="B633">
-        <v>885169</v>
+        <v>888742</v>
       </c>
       <c r="C633">
         <v>1399.5</v>
       </c>
       <c r="D633">
-        <v>355131</v>
+        <v>356591</v>
       </c>
       <c r="E633">
-        <v>120402</v>
+        <v>118733</v>
       </c>
       <c r="F633">
-        <v>6362974</v>
+        <v>6337806</v>
       </c>
       <c r="G633">
-        <v>5288548</v>
+        <v>5273207</v>
       </c>
       <c r="H633">
-        <v>2005155</v>
+        <v>2003703</v>
       </c>
       <c r="I633">
-        <v>389.96</v>
+        <v>390.7</v>
       </c>
       <c r="J633">
-        <v>30.26</v>
+        <v>30.24</v>
       </c>
       <c r="K633">
-        <v>15.63</v>
+        <v>15.62</v>
       </c>
       <c r="L633">
-        <v>382.63</v>
+        <v>382.69</v>
       </c>
       <c r="M633">
-        <v>26097068</v>
+        <v>26095610</v>
       </c>
       <c r="N633">
-        <v>4536460</v>
+        <v>4537909</v>
       </c>
       <c r="O633">
-        <v>2081069</v>
+        <v>2079339</v>
       </c>
       <c r="P633">
         <v>5261</v>
@@ -33960,52 +33960,52 @@
         <v>44834</v>
       </c>
       <c r="B634">
-        <v>718568</v>
+        <v>724096</v>
       </c>
       <c r="C634">
         <v>1218.6</v>
       </c>
       <c r="D634">
-        <v>286050</v>
+        <v>286277</v>
       </c>
       <c r="E634">
-        <v>106776</v>
+        <v>101927</v>
       </c>
       <c r="F634">
-        <v>5707588</v>
+        <v>5688799</v>
       </c>
       <c r="G634">
-        <v>4188330</v>
+        <v>4175701</v>
       </c>
       <c r="H634">
-        <v>1653091</v>
+        <v>1653357</v>
       </c>
       <c r="I634">
-        <v>403.73</v>
+        <v>404.74</v>
       </c>
       <c r="J634">
-        <v>29.42</v>
+        <v>29.32</v>
       </c>
       <c r="K634">
-        <v>15.42</v>
+        <v>15.41</v>
       </c>
       <c r="L634">
-        <v>387.52</v>
+        <v>387.64</v>
       </c>
       <c r="M634">
-        <v>25066164</v>
+        <v>25064971</v>
       </c>
       <c r="N634">
-        <v>4344323</v>
+        <v>4345999</v>
       </c>
       <c r="O634">
-        <v>1882229</v>
+        <v>1875650</v>
       </c>
       <c r="P634">
-        <v>5261</v>
+        <v>5273</v>
       </c>
       <c r="Q634">
-        <v>14194</v>
+        <v>14200</v>
       </c>
       <c r="R634">
         <v>348166</v>
@@ -34015,17 +34015,67 @@
       <c r="A635" s="2">
         <v>44865</v>
       </c>
+      <c r="B635">
+        <v>826695</v>
+      </c>
       <c r="C635">
         <v>1222.3</v>
       </c>
+      <c r="D635">
+        <v>294264</v>
+      </c>
+      <c r="E635">
+        <v>114228</v>
+      </c>
+      <c r="F635">
+        <v>5627721</v>
+      </c>
+      <c r="G635">
+        <v>4359116</v>
+      </c>
+      <c r="H635">
+        <v>1732508</v>
+      </c>
+      <c r="I635">
+        <v>407.33</v>
+      </c>
+      <c r="J635">
+        <v>29.88</v>
+      </c>
+      <c r="K635">
+        <v>15.06</v>
+      </c>
+      <c r="L635">
+        <v>392.77</v>
+      </c>
+      <c r="M635">
+        <v>24541990</v>
+      </c>
+      <c r="N635">
+        <v>4286306</v>
+      </c>
+      <c r="O635">
+        <v>1683902</v>
+      </c>
       <c r="P635">
-        <v>5254</v>
+        <v>5273</v>
       </c>
       <c r="Q635">
-        <v>14223</v>
+        <v>14231</v>
       </c>
       <c r="R635">
         <v>348475</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2">
+        <v>44895</v>
+      </c>
+      <c r="P636">
+        <v>5284</v>
+      </c>
+      <c r="Q636">
+        <v>14263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>